<commit_message>
chore: refresh competitor intelligence (all)
</commit_message>
<xml_diff>
--- a/competitor_campaigns_latest.xlsx
+++ b/competitor_campaigns_latest.xlsx
@@ -4633,7 +4633,7 @@
         <x:v>Research Cut-off</x:v>
       </x:c>
       <x:c r="B3" s="227" t="n">
-        <x:v>46277.88188063022</x:v>
+        <x:v>46277.986707524535</x:v>
       </x:c>
       <x:c r="C3" s="227"/>
       <x:c r="D3" s="227"/>
@@ -4648,7 +4648,7 @@
         <x:v>Status As Of</x:v>
       </x:c>
       <x:c r="K3" s="227" t="n">
-        <x:v>46277.883267949794</x:v>
+        <x:v>46277.99069170773</x:v>
       </x:c>
       <x:c r="L3" s="227"/>
       <x:c r="M3" s="227"/>
@@ -8038,7 +8038,7 @@
       <x:c r="L4" s="43"/>
       <x:c r="M4" s="44" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Merchant Offers (Count Only): 68</x:t>
+          <x:t xml:space="preserve">Merchant Offers (Count Only): 62</x:t>
         </x:is>
       </x:c>
       <x:c r="N4" s="44"/>

</xml_diff>